<commit_message>
feat: add Sex to student import and make SF2 computations accurate
Student/SHS import now accepts a Sex column (Male/Female dropdown in
the XLSX templates, validated on preview, stored on insert and update;
existing gender is kept when the file omits it).

SF2 accuracy fixes:
- future school days are no longer marked or counted as absences; a
  day only counts after it ends (absence_cutoff_time setting), the
  same rule the attendance API uses
- holidays and manual school-day overrides are excluded from the grid
  and all totals; the date grid is built TZ-safe (no UTC day shift)
- gender grouping is case-insensitive (m/male/M all match); students
  without a sex are listed separately with a SEX NOT SET remark
  instead of silently landing under FEMALE
- summary box now computes real values: enrolment as of first Friday,
  late enrolment during the month, 5-consecutive-day absences per
  sex, and guarded percentage formulas (no divide-by-zero)
</commit_message>
<xml_diff>
--- a/public/templates/shs_student_import_template.xlsx
+++ b/public/templates/shs_student_import_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
   <si>
     <r>
       <rPr>
@@ -58,6 +58,25 @@
         <color rgb="FFFFFFFF"/>
         <sz val="11"/>
       </rPr>
+      <t xml:space="preserve">Sex
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="9"/>
+      </rPr>
+      <t>((Select from dropdown))</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+      </rPr>
       <t xml:space="preserve">School
 </t>
     </r>
@@ -162,6 +181,9 @@
     <t>7</t>
   </si>
   <si>
+    <t>Male</t>
+  </si>
+  <si>
     <t>Banag Elementary School</t>
   </si>
   <si>
@@ -175,6 +197,9 @@
   </si>
   <si>
     <t>8</t>
+  </si>
+  <si>
+    <t>Female</t>
   </si>
   <si>
     <t>Barangay V Elementary School</t>
@@ -745,19 +770,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -779,125 +805,134 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="3:5" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="3:5" x14ac:dyDescent="0.25"/>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="3:6" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select School" prompt="Choose from the list" sqref="C10:C101">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Sex" prompt="Choose from the list" sqref="C10:C101">
+      <formula1>Dropdowns!$H$1:$H$2</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Sex" prompt="Choose from the list" sqref="C2:C101">
+      <formula1>Dropdowns!$H$1:$H$2</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select School" prompt="Choose from the list" sqref="D10:D101">
       <formula1>Dropdowns!$A$1:$A$45</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select School" prompt="Choose from the list" sqref="C2:C101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select School" prompt="Choose from the list" sqref="D2:D101">
       <formula1>Dropdowns!$A$1:$A$45</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="D10:D101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="E10:E101">
       <formula1>Dropdowns!$B$1:$B$12</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="D2:D101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="E2:E101">
       <formula1>Dropdowns!$B$1:$B$12</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Track" prompt="Choose from the list" sqref="E10:E101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Track" prompt="Choose from the list" sqref="F10:F101">
       <formula1>Dropdowns!$C$1:$C$10</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Track" prompt="Choose from the list" sqref="E2:E101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Track" prompt="Choose from the list" sqref="F2:F101">
       <formula1>Dropdowns!$C$1:$C$10</formula1>
     </dataValidation>
   </dataValidations>
@@ -908,469 +943,475 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
-      </c>
       <c r="G1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
       <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E17" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D22" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D23" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D26" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: remove blank grade options from student templates
</commit_message>
<xml_diff>
--- a/public/templates/shs_student_import_template.xlsx
+++ b/public/templates/shs_student_import_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="77">
   <si>
     <r>
       <rPr>
@@ -169,15 +169,18 @@
     <t>Agripino Alvarez Elementary School</t>
   </si>
   <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>STEM</t>
+  </si>
+  <si>
+    <t>Cambogui-ot National High School</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
-    <t>STEM</t>
-  </si>
-  <si>
-    <t>Cambogui-ot National High School</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
@@ -187,15 +190,18 @@
     <t>Banag Elementary School</t>
   </si>
   <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>ABM</t>
+  </si>
+  <si>
+    <t>Camindangan National High School</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
-    <t>ABM</t>
-  </si>
-  <si>
-    <t>Camindangan National High School</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -205,61 +211,55 @@
     <t>Barangay V Elementary School</t>
   </si>
   <si>
+    <t>HUMSS</t>
+  </si>
+  <si>
+    <t>Cayhagan National High School</t>
+  </si>
+  <si>
     <t>3</t>
   </si>
   <si>
-    <t>HUMSS</t>
-  </si>
-  <si>
-    <t>Cayhagan National High School</t>
-  </si>
-  <si>
     <t>9</t>
   </si>
   <si>
     <t>Barasbarasan Elementary School</t>
   </si>
   <si>
+    <t>GAS</t>
+  </si>
+  <si>
+    <t>Dung-i Integrated School</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
-    <t>GAS</t>
-  </si>
-  <si>
-    <t>Dung-i Integrated School</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
     <t>Bawog Elementary School</t>
   </si>
   <si>
+    <t>TVL-HE</t>
+  </si>
+  <si>
+    <t>Dungga Integrated School</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
-    <t>TVL-HE</t>
-  </si>
-  <si>
-    <t>Dungga Integrated School</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
     <t>Binotusan Elementary School</t>
   </si>
   <si>
+    <t>TVL-ICT</t>
+  </si>
+  <si>
+    <t>Gil Montilla National High School</t>
+  </si>
+  <si>
     <t>6</t>
-  </si>
-  <si>
-    <t>TVL-ICT</t>
-  </si>
-  <si>
-    <t>Gil Montilla National High School</t>
-  </si>
-  <si>
-    <t>12</t>
   </si>
   <si>
     <t>Binulig Elementary School</t>
@@ -924,10 +924,10 @@
       <formula1>Dropdowns!$A$1:$A$45</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="E10:E101">
-      <formula1>Dropdowns!$B$1:$B$12</formula1>
+      <formula1>Dropdowns!$B$1:$B$2</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Grade" prompt="Choose from the list" sqref="E2:E101">
-      <formula1>Dropdowns!$B$1:$B$12</formula1>
+      <formula1>Dropdowns!$B$1:$B$2</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Track" prompt="Choose from the list" sqref="F10:F101">
       <formula1>Dropdowns!$C$1:$C$10</formula1>
@@ -963,140 +963,125 @@
         <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
-        <v>25</v>
-      </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
-        <v>30</v>
-      </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" t="s">
         <v>36</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
         <v>38</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
       <c r="C7" t="s">
         <v>41</v>
       </c>
@@ -1111,9 +1096,6 @@
       <c r="A8" t="s">
         <v>43</v>
       </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
       <c r="C8" t="s">
         <v>44</v>
       </c>
@@ -1128,9 +1110,6 @@
       <c r="A9" t="s">
         <v>46</v>
       </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
       <c r="C9" t="s">
         <v>47</v>
       </c>
@@ -1145,9 +1124,6 @@
       <c r="A10" t="s">
         <v>49</v>
       </c>
-      <c r="B10" t="s">
-        <v>29</v>
-      </c>
       <c r="C10" t="s">
         <v>50</v>
       </c>
@@ -1162,9 +1138,6 @@
       <c r="A11" t="s">
         <v>52</v>
       </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
       <c r="D11" t="s">
         <v>52</v>
       </c>
@@ -1176,9 +1149,6 @@
       <c r="A12" t="s">
         <v>54</v>
       </c>
-      <c r="B12" t="s">
-        <v>39</v>
-      </c>
       <c r="D12" t="s">
         <v>54</v>
       </c>
@@ -1210,7 +1180,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
         <v>60</v>
@@ -1267,7 +1237,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D21" t="s">
         <v>69</v>
@@ -1283,7 +1253,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
         <v>71</v>
@@ -1291,7 +1261,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D24" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
fix: preserve leading zeros in import templates
</commit_message>
<xml_diff>
--- a/public/templates/shs_student_import_template.xlsx
+++ b/public/templates/shs_student_import_template.xlsx
@@ -426,8 +426,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -773,142 +777,442 @@
   <dimension ref="A1:H101"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="22" style="1" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="3:6" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="H10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="H12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="H18" s="1"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="H20" s="1"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="H24" s="1"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="H25" s="1"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="H27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="H28" s="1"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="H29" s="1"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="H31" s="1"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="H33" s="1"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="H34" s="1"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="H38" s="1"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="1"/>
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+      <c r="H42" s="1"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="1"/>
+      <c r="H43" s="1"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="1"/>
+      <c r="H44" s="1"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="1"/>
+      <c r="H45" s="1"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="1"/>
+      <c r="H46" s="1"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="1"/>
+      <c r="H47" s="1"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="1"/>
+      <c r="H48" s="1"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="1"/>
+      <c r="H49" s="1"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="1"/>
+      <c r="H50" s="1"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="1"/>
+      <c r="H51" s="1"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="1"/>
+      <c r="H52" s="1"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="1"/>
+      <c r="H53" s="1"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="1"/>
+      <c r="H54" s="1"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="1"/>
+      <c r="H55" s="1"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="1"/>
+      <c r="H56" s="1"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="1"/>
+      <c r="H57" s="1"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="1"/>
+      <c r="H58" s="1"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="1"/>
+      <c r="H59" s="1"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="1"/>
+      <c r="H60" s="1"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="1"/>
+      <c r="H61" s="1"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="1"/>
+      <c r="H62" s="1"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="1"/>
+      <c r="H63" s="1"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="1"/>
+      <c r="H64" s="1"/>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" s="1"/>
+      <c r="H65" s="1"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="1"/>
+      <c r="H66" s="1"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="1"/>
+      <c r="H67" s="1"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="1"/>
+      <c r="H68" s="1"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" s="1"/>
+      <c r="H69" s="1"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="1"/>
+      <c r="H70" s="1"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="1"/>
+      <c r="H71" s="1"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" s="1"/>
+      <c r="H72" s="1"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" s="1"/>
+      <c r="H73" s="1"/>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74" s="1"/>
+      <c r="H74" s="1"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" s="1"/>
+      <c r="H75" s="1"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" s="1"/>
+      <c r="H76" s="1"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="1"/>
+      <c r="H77" s="1"/>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="1"/>
+      <c r="H78" s="1"/>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="1"/>
+      <c r="H79" s="1"/>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="1"/>
+      <c r="H80" s="1"/>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="1"/>
+      <c r="H81" s="1"/>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="1"/>
+      <c r="H82" s="1"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="1"/>
+      <c r="H83" s="1"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" s="1"/>
+      <c r="H84" s="1"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="1"/>
+      <c r="H85" s="1"/>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" s="1"/>
+      <c r="H86" s="1"/>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" s="1"/>
+      <c r="H87" s="1"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="1"/>
+      <c r="H88" s="1"/>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="1"/>
+      <c r="H89" s="1"/>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" s="1"/>
+      <c r="H90" s="1"/>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" s="1"/>
+      <c r="H91" s="1"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="1"/>
+      <c r="H92" s="1"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="1"/>
+      <c r="H93" s="1"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="1"/>
+      <c r="H94" s="1"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="1"/>
+      <c r="H95" s="1"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="1"/>
+      <c r="H96" s="1"/>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" s="1"/>
+      <c r="H97" s="1"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" s="1"/>
+      <c r="H98" s="1"/>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" s="1"/>
+      <c r="H99" s="1"/>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" s="1"/>
+      <c r="H100" s="1"/>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" s="1"/>
+      <c r="H101" s="1"/>
+    </row>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Select Sex" prompt="Choose from the list" sqref="C10:C101">

</xml_diff>